<commit_message>
4808 - Data for MOQ by BOE by Task sheet of Excel export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBAA886-7FC9-4148-9EFB-AD5BDAE38AED}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD718BDA-BCC8-4FBD-9694-69CA25128284}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,9 +52,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId19"/>
-    <pivotCache cacheId="10" r:id="rId20"/>
-    <pivotCache cacheId="11" r:id="rId21"/>
+    <pivotCache cacheId="54" r:id="rId19"/>
+    <pivotCache cacheId="55" r:id="rId20"/>
+    <pivotCache cacheId="56" r:id="rId21"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4230,7 +4230,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="54" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4579,7 +4579,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4788,7 +4788,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="56" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -8884,6 +8884,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -8986,19 +8999,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
@@ -9008,6 +9008,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9024,21 +9041,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4957 - Remove the Total WBS/WBS Element Hours for SSC
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDD0106-7D79-4634-88B3-66DDF8F23CC6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC460066-7B75-41A0-9A23-5EAAC30EEF42}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
@@ -52,9 +52,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="30" r:id="rId19"/>
-    <pivotCache cacheId="31" r:id="rId20"/>
-    <pivotCache cacheId="32" r:id="rId21"/>
+    <pivotCache cacheId="0" r:id="rId19"/>
+    <pivotCache cacheId="1" r:id="rId20"/>
+    <pivotCache cacheId="2" r:id="rId21"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -319,7 +319,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="143">
   <si>
     <t>Start Date</t>
   </si>
@@ -736,9 +736,6 @@
   </si>
   <si>
     <t>WBS/WBS Element</t>
-  </si>
-  <si>
-    <t>Total WBS/WBS Element Hours</t>
   </si>
   <si>
     <t>Additional Query Filters (i.e. cost number, employee id)</t>
@@ -4232,7 +4229,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="30" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4581,7 +4578,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="31" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4790,7 +4787,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="32" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6115,7 +6112,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB92274E-9194-432C-BABA-DBDF288E7F50}">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6131,12 +6128,11 @@
     <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="42" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="61.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6182,13 +6178,10 @@
       <c r="O1" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="P1" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:P1" xr:uid="{9A7F204E-ACEF-43F5-B840-26856445FC24}"/>
+  <autoFilter ref="A1:O1" xr:uid="{9A7F204E-ACEF-43F5-B840-26856445FC24}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6208,10 +6201,10 @@
         <v>85</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="39" t="s">
         <v>142</v>
-      </c>
-      <c r="C1" s="39" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -8873,6 +8866,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -8975,29 +8990,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9014,29 +9032,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4962/4963 - Updates to Additional Query Filters
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDD0106-7D79-4634-88B3-66DDF8F23CC6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEC9F69-AFB5-44C1-AA6D-16B260EF9879}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="345" windowWidth="18900" windowHeight="11055" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -52,9 +52,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="30" r:id="rId19"/>
-    <pivotCache cacheId="31" r:id="rId20"/>
-    <pivotCache cacheId="32" r:id="rId21"/>
+    <pivotCache cacheId="0" r:id="rId19"/>
+    <pivotCache cacheId="1" r:id="rId20"/>
+    <pivotCache cacheId="2" r:id="rId21"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -741,16 +741,16 @@
     <t>Total WBS/WBS Element Hours</t>
   </si>
   <si>
-    <t>Additional Query Filters (i.e. cost number, employee id)</t>
-  </si>
-  <si>
-    <t>Total Relevant Hours After Additional Query Filters Applied</t>
-  </si>
-  <si>
     <t>MOQ Hours Bid/Spread</t>
   </si>
   <si>
     <t>% of total</t>
+  </si>
+  <si>
+    <t>Employee ID Filters</t>
+  </si>
+  <si>
+    <t>Total Relevant Hours After Employee ID Filters Applied</t>
   </si>
 </sst>
 </file>
@@ -4232,7 +4232,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="30" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4581,7 +4581,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="31" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4790,7 +4790,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="32" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6180,10 +6180,10 @@
         <v>139</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6208,10 +6208,10 @@
         <v>85</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C1" s="39" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -8873,6 +8873,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -8975,29 +8997,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9014,29 +9039,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates to make sure the percentages are correct when exporting and retrieving from database
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e309214\source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBEA335-0BD0-483F-946D-A300EB09BC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC7E66A-090D-4261-A63C-06A6D427DEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19395" windowHeight="15480" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -24,8 +24,8 @@
     <sheet name="Resource Spreads" sheetId="41" r:id="rId9"/>
     <sheet name="MOQ by BOE by Task" sheetId="43" r:id="rId10"/>
     <sheet name="MOQ Table Data" sheetId="44" r:id="rId11"/>
-    <sheet name="Current Skill Mix" sheetId="46" r:id="rId12"/>
-    <sheet name="Common Disclosure Skill Mix" sheetId="45" r:id="rId13"/>
+    <sheet name="Legacy Skill Mix" sheetId="46" r:id="rId12"/>
+    <sheet name="LM Enterprise Skill Mix" sheetId="45" r:id="rId13"/>
     <sheet name="WBS" sheetId="24" r:id="rId14"/>
     <sheet name="User Permissions" sheetId="39" r:id="rId15"/>
     <sheet name="CLINs" sheetId="25" r:id="rId16"/>
@@ -40,8 +40,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Common Disclosure Skill Mix'!$A$1:$N$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Current Skill Mix'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Legacy Skill Mix'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'LM Enterprise Skill Mix'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$B$1:$Q$2</definedName>
@@ -55,9 +55,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId20"/>
-    <pivotCache cacheId="13" r:id="rId21"/>
-    <pivotCache cacheId="14" r:id="rId22"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="1" r:id="rId21"/>
+    <pivotCache cacheId="2" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4289,7 +4289,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4638,7 +4638,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4847,7 +4847,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -9131,28 +9131,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9255,10 +9233,43 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9281,20 +9292,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated excel sheet and exporter
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\IES\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e426263\source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96088262-8478-48E8-A7D8-ED2D92AC6608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34083DD1-6AF8-428E-8120-B3C2519D84A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15105" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -36,7 +36,7 @@
     <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AV$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AW$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
@@ -55,9 +55,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="48" r:id="rId20"/>
-    <pivotCache cacheId="49" r:id="rId21"/>
-    <pivotCache cacheId="50" r:id="rId22"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="1" r:id="rId21"/>
+    <pivotCache cacheId="2" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -322,7 +322,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="159">
   <si>
     <t>Start Date</t>
   </si>
@@ -4289,7 +4289,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="48" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4638,7 +4638,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="49" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4847,7 +4847,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="50" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -8554,7 +8554,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" customWidth="1"/>
@@ -8598,12 +8598,13 @@
     <col min="44" max="44" width="8.7109375" style="38" customWidth="1"/>
     <col min="45" max="45" width="10.5703125" style="38" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="10" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="14.7109375" style="44" customWidth="1"/>
-    <col min="48" max="48" width="9.140625" style="29"/>
-    <col min="49" max="16384" width="9.140625" style="1"/>
+    <col min="47" max="47" width="16.140625" style="44" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="16.140625" style="44" customWidth="1"/>
+    <col min="49" max="49" width="9.140625" style="29"/>
+    <col min="50" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8745,13 +8746,16 @@
       <c r="AU1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="AV1" s="27" t="s">
+      <c r="AV1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="AW1" s="27" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:48" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:49" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AV2" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
+  <autoFilter ref="A1:AW2" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9126,28 +9130,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9250,10 +9232,43 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9276,20 +9291,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update excel sheet open location
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e426263\source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34083DD1-6AF8-428E-8120-B3C2519D84A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13764607-55C8-4153-9C9D-2B561F791C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14025" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -9130,6 +9130,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9232,43 +9254,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9291,9 +9280,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update workspace data export for Space to show Skill Mix Summary sheet and not the older 2 sheets
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D82D017-A0B6-46B0-867F-A9EE31C5A497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C551256-D243-4F3B-BD62-711C3C5C6A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15510" yWindow="0" windowWidth="19410" windowHeight="15480" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -24,27 +24,25 @@
     <sheet name="Resource Spreads" sheetId="41" r:id="rId9"/>
     <sheet name="MOQ by BOE by Task" sheetId="43" r:id="rId10"/>
     <sheet name="MOQ Table Data" sheetId="44" r:id="rId11"/>
-    <sheet name="Legacy Skill Mix" sheetId="46" r:id="rId12"/>
-    <sheet name="LM Enterprise Skill Mix" sheetId="45" r:id="rId13"/>
-    <sheet name="WBS" sheetId="24" r:id="rId14"/>
-    <sheet name="User Permissions" sheetId="39" r:id="rId15"/>
-    <sheet name="CLINs" sheetId="25" r:id="rId16"/>
-    <sheet name="Workspace Identification" sheetId="40" r:id="rId17"/>
+    <sheet name="Skill Mix Summary" sheetId="45" r:id="rId12"/>
+    <sheet name="WBS" sheetId="24" r:id="rId13"/>
+    <sheet name="User Permissions" sheetId="39" r:id="rId14"/>
+    <sheet name="CLINs" sheetId="25" r:id="rId15"/>
+    <sheet name="Workspace Identification" sheetId="40" r:id="rId16"/>
   </sheets>
   <externalReferences>
+    <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
-    <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AW$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Legacy Skill Mix'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'LM Enterprise Skill Mix'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$B$1:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Skill Mix Summary'!$A$1:$Q$1</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
     <definedName name="CLINs">'[1]Options Lists'!$B$2:$B$5</definedName>
@@ -55,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="0" r:id="rId19"/>
+    <pivotCache cacheId="1" r:id="rId20"/>
+    <pivotCache cacheId="2" r:id="rId21"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -322,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="159">
   <si>
     <t>Start Date</t>
   </si>
@@ -768,27 +766,9 @@
     <t>Historical Hours</t>
   </si>
   <si>
-    <t>Labor Skill Mix</t>
-  </si>
-  <si>
-    <t>Included</t>
-  </si>
-  <si>
-    <t>BOE Skill Mix</t>
-  </si>
-  <si>
-    <t>Proposed Hours</t>
-  </si>
-  <si>
     <t>Rationale </t>
   </si>
   <si>
-    <t xml:space="preserve">Included </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current Resource	</t>
-  </si>
-  <si>
     <t>Current Resource</t>
   </si>
   <si>
@@ -799,19 +779,36 @@
   </si>
   <si>
     <t>Task Author</t>
+  </si>
+  <si>
+    <t>Historical Skill Mix</t>
+  </si>
+  <si>
+    <t>Proposed Skill Mix</t>
+  </si>
+  <si>
+    <t>Proposed Legacy Resource</t>
+  </si>
+  <si>
+    <t>Proposed BRC</t>
+  </si>
+  <si>
+    <t>Total Proposed Legacy &amp; BRC</t>
+  </si>
+  <si>
+    <t>Grand Total Hours</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -979,7 +976,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -1085,10 +1082,6 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -6238,77 +6231,8 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC859F52-06EC-4D10-BF03-A04146FE2305}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" style="40" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17" style="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.28515625" style="43" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H1" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="I1" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="K1" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="L1" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{BC859F52-06EC-4D10-BF03-A04146FE2305}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF11AB7-F45F-4865-B8BC-DBCCDB5DD031}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6320,14 +6244,15 @@
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.7109375" style="40" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" style="33" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="43" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" style="33" customWidth="1"/>
+    <col min="11" max="11" width="22.140625" style="33" customWidth="1"/>
+    <col min="12" max="12" width="29.28515625" style="42" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="29.5703125" style="41" customWidth="1"/>
+    <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6347,38 +6272,47 @@
         <v>85</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I1" s="39" t="s">
         <v>147</v>
       </c>
       <c r="J1" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="K1" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="O1" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="P1" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="L1" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="M1" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{5AF11AB7-F45F-4865-B8BC-DBCCDB5DD031}"/>
+  <autoFilter ref="A1:Q1" xr:uid="{5AF11AB7-F45F-4865-B8BC-DBCCDB5DD031}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:E2"/>
@@ -6419,7 +6353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:I2"/>
@@ -6476,7 +6410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:F2"/>
@@ -6522,7 +6456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="A1:A18"/>
@@ -8599,8 +8533,8 @@
     <col min="44" max="44" width="8.7109375" style="38" customWidth="1"/>
     <col min="45" max="45" width="10.5703125" style="38" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="10" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="16.140625" style="44" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="16.140625" style="44" customWidth="1"/>
+    <col min="47" max="47" width="16.140625" style="42" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="16.140625" style="42" customWidth="1"/>
     <col min="49" max="49" width="9.140625" style="29"/>
     <col min="50" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -8625,7 +8559,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>122</v>
@@ -8745,7 +8679,7 @@
         <v>110</v>
       </c>
       <c r="AU1" s="5" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="AV1" s="5" t="s">
         <v>6</v>
@@ -8868,7 +8802,7 @@
         <v>84</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>122</v>
@@ -9135,28 +9069,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9259,32 +9171,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9301,4 +9210,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Make changes for commas to UAT
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Code Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C551256-D243-4F3B-BD62-711C3C5C6A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90436C3F-DCDE-443C-9A0B-913A2BB8CDDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15510" yWindow="0" windowWidth="19410" windowHeight="15480" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -803,12 +803,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1078,14 +1077,14 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -6243,12 +6242,12 @@
     <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" style="40" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7109375" style="41" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.140625" style="33" customWidth="1"/>
     <col min="11" max="11" width="22.140625" style="33" customWidth="1"/>
-    <col min="12" max="12" width="29.28515625" style="42" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="29.5703125" style="41" customWidth="1"/>
+    <col min="12" max="12" width="29.28515625" style="41" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" style="42" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="29.5703125" style="42" customWidth="1"/>
     <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6277,7 +6276,7 @@
       <c r="H1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="I1" s="39" t="s">
+      <c r="I1" s="40" t="s">
         <v>147</v>
       </c>
       <c r="J1" s="32" t="s">
@@ -6286,19 +6285,19 @@
       <c r="K1" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="L1" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="N1" s="19" t="s">
+      <c r="N1" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="O1" s="19" t="s">
+      <c r="O1" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="40" t="s">
         <v>158</v>
       </c>
       <c r="Q1" s="5" t="s">
@@ -8533,8 +8532,8 @@
     <col min="44" max="44" width="8.7109375" style="38" customWidth="1"/>
     <col min="45" max="45" width="10.5703125" style="38" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="10" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="16.140625" style="42" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="16.140625" style="42" customWidth="1"/>
+    <col min="47" max="47" width="16.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="16.140625" style="39" customWidth="1"/>
     <col min="49" max="49" width="9.140625" style="29"/>
     <col min="50" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -9172,15 +9171,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -9191,6 +9181,15 @@
     </SipLabel>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9213,14 +9212,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9235,4 +9226,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
remove from rms and update template
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataSpaceSystems.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Code Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e402751\Project\FB&amp;I\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{810E7EBD-C9E0-4920-95DE-E2396B44CD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF797106-F36B-4301-B92D-7A75E3933144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1250" yWindow="1130" windowWidth="17060" windowHeight="8660" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -53,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId19"/>
-    <pivotCache cacheId="1" r:id="rId20"/>
-    <pivotCache cacheId="2" r:id="rId21"/>
+    <pivotCache cacheId="6" r:id="rId19"/>
+    <pivotCache cacheId="7" r:id="rId20"/>
+    <pivotCache cacheId="8" r:id="rId21"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="160">
   <si>
     <t>Start Date</t>
   </si>
@@ -797,6 +797,9 @@
   </si>
   <si>
     <t>Grand Total Hours</t>
+  </si>
+  <si>
+    <t>Current Workspace</t>
   </si>
 </sst>
 </file>
@@ -4281,7 +4284,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4630,7 +4633,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4839,7 +4842,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -5570,25 +5573,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A3:N32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" customWidth="1"/>
+    <col min="3" max="3" width="10.54296875" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>33</v>
       </c>
@@ -5632,7 +5635,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -5676,7 +5679,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G6" t="s">
         <v>57</v>
       </c>
@@ -5702,7 +5705,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H8" t="s">
         <v>43</v>
       </c>
@@ -5725,7 +5728,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="D10" t="s">
         <v>62</v>
       </c>
@@ -5760,7 +5763,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G12" t="s">
         <v>57</v>
       </c>
@@ -5786,7 +5789,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H14" t="s">
         <v>43</v>
       </c>
@@ -5809,7 +5812,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
         <v>57</v>
       </c>
@@ -5844,7 +5847,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -5888,7 +5891,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G20" t="s">
         <v>57</v>
       </c>
@@ -5914,7 +5917,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H22" t="s">
         <v>43</v>
       </c>
@@ -5937,7 +5940,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H24" t="s">
         <v>55</v>
       </c>
@@ -5960,7 +5963,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H26" t="s">
         <v>51</v>
       </c>
@@ -5983,7 +5986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="D28" t="s">
         <v>64</v>
       </c>
@@ -6018,7 +6021,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G30" t="s">
         <v>57</v>
       </c>
@@ -6044,7 +6047,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="D32" t="s">
         <v>62</v>
       </c>
@@ -6092,18 +6095,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE13AD99-C0B6-4E90-ABF6-10E14BCDEE02}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.26953125" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="64.140625" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="64.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6129,7 +6132,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{9706A812-64F4-4103-BF42-450B5D5EA342}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6143,28 +6146,28 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB92274E-9194-432C-BABA-DBDF288E7F50}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.26953125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" style="1" customWidth="1"/>
-    <col min="6" max="6" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="42" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="41.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="56.5703125" style="31" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="56.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.453125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="5" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6217,7 +6220,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:P1" xr:uid="{B03D36E4-F111-482D-8BA5-A875D16A6E86}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6232,26 +6235,26 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF11AB7-F45F-4865-B8BC-DBCCDB5DD031}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" style="41" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.140625" style="33" customWidth="1"/>
-    <col min="11" max="11" width="22.140625" style="33" customWidth="1"/>
-    <col min="12" max="12" width="29.28515625" style="41" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="42" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="29.5703125" style="42" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.1796875" style="33" customWidth="1"/>
+    <col min="11" max="11" width="22.1796875" style="33" customWidth="1"/>
+    <col min="12" max="12" width="29.26953125" style="41" customWidth="1"/>
+    <col min="13" max="13" width="19.26953125" style="42" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="29.54296875" style="42" customWidth="1"/>
     <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6304,7 +6307,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{5AF11AB7-F45F-4865-B8BC-DBCCDB5DD031}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6316,15 +6319,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="4" width="30.7109375" style="8" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="30.7265625" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="30.7265625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.1796875" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>68</v>
       </c>
@@ -6341,7 +6344,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6357,20 +6360,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="15" customWidth="1"/>
-    <col min="2" max="3" width="35.7109375" style="15" customWidth="1"/>
-    <col min="4" max="4" width="26.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="15"/>
+    <col min="1" max="1" width="18.81640625" style="15" customWidth="1"/>
+    <col min="2" max="3" width="35.7265625" style="15" customWidth="1"/>
+    <col min="4" max="4" width="26.1796875" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.1796875" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.81640625" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.1796875" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="14" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="14" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>71</v>
       </c>
@@ -6399,7 +6402,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6414,17 +6417,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="50.7109375" style="8" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" style="8" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="7" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="13.1796875" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7265625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="50.7265625" style="8" customWidth="1"/>
+    <col min="4" max="5" width="20.7265625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" style="7" customWidth="1"/>
+    <col min="7" max="16384" width="9.1796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>98</v>
       </c>
@@ -6444,7 +6447,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6459,98 +6462,103 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1:A18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="32.26953125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="82.1796875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="10" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -6567,28 +6575,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="13.5703125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="3"/>
+    <col min="15" max="17" width="13.54296875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
@@ -6632,7 +6640,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>59</v>
       </c>
@@ -6643,7 +6651,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>59</v>
       </c>
@@ -6666,7 +6674,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
@@ -6707,7 +6715,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>59</v>
       </c>
@@ -6748,7 +6756,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>59</v>
       </c>
@@ -6771,7 +6779,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>59</v>
       </c>
@@ -6812,7 +6820,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -6853,7 +6861,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>60</v>
       </c>
@@ -6873,7 +6881,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>60</v>
       </c>
@@ -6896,7 +6904,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -6937,7 +6945,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>60</v>
       </c>
@@ -6978,7 +6986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>60</v>
       </c>
@@ -7019,7 +7027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>60</v>
       </c>
@@ -7060,7 +7068,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>60</v>
       </c>
@@ -7083,7 +7091,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>60</v>
       </c>
@@ -7139,20 +7147,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A3:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.54296875" customWidth="1"/>
+    <col min="2" max="2" width="8.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="8" max="8" width="9.453125" customWidth="1"/>
     <col min="9" max="19" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -7178,7 +7186,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -7204,7 +7212,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>45</v>
       </c>
@@ -7212,7 +7220,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7238,12 +7246,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="H7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>45</v>
       </c>
@@ -7251,7 +7259,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -7277,12 +7285,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="H10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>45</v>
       </c>
@@ -7304,29 +7312,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A3:T32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -7388,7 +7396,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -7450,7 +7458,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -7509,7 +7517,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="I8" t="s">
         <v>40</v>
       </c>
@@ -7547,7 +7555,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -7606,7 +7614,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="R12" t="s">
         <v>20</v>
       </c>
@@ -7617,7 +7625,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="N14" t="s">
         <v>43</v>
       </c>
@@ -7640,7 +7648,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="O16" t="s">
         <v>53</v>
       </c>
@@ -7660,7 +7668,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -7722,7 +7730,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>34</v>
       </c>
@@ -7781,7 +7789,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="I22" t="s">
         <v>49</v>
       </c>
@@ -7819,7 +7827,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>12</v>
       </c>
@@ -7878,7 +7886,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="O26" t="s">
         <v>52</v>
       </c>
@@ -7898,7 +7906,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="N28" t="s">
         <v>43</v>
       </c>
@@ -7921,7 +7929,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="N30" t="s">
         <v>55</v>
       </c>
@@ -7944,7 +7952,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="N32" t="s">
         <v>51</v>
       </c>
@@ -7981,33 +7989,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="3"/>
-    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" style="3"/>
+    <col min="2" max="3" width="10.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="13.5703125" style="3" customWidth="1"/>
-    <col min="24" max="24" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.140625" style="3"/>
+    <col min="21" max="23" width="13.54296875" style="3" customWidth="1"/>
+    <col min="24" max="24" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
@@ -8069,7 +8077,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
@@ -8095,7 +8103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -8118,7 +8126,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -8147,7 +8155,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>58</v>
       </c>
@@ -8176,7 +8184,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>58</v>
       </c>
@@ -8199,7 +8207,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -8228,7 +8236,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>58</v>
       </c>
@@ -8257,7 +8265,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>45</v>
       </c>
@@ -8283,7 +8291,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
@@ -8306,7 +8314,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
@@ -8335,7 +8343,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
@@ -8364,7 +8372,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>45</v>
       </c>
@@ -8393,7 +8401,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>45</v>
       </c>
@@ -8422,7 +8430,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>45</v>
       </c>
@@ -8445,7 +8453,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>45</v>
       </c>
@@ -8489,57 +8497,57 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:AW2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="13.42578125" style="36" customWidth="1"/>
-    <col min="18" max="18" width="12.5703125" style="36" customWidth="1"/>
-    <col min="19" max="19" width="21.42578125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="20.140625" style="31" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.7109375" style="36" customWidth="1"/>
-    <col min="25" max="25" width="12.85546875" style="36" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.7109375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="31" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="1" customWidth="1"/>
+    <col min="3" max="4" width="15.7265625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="19.1796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.81640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.54296875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.54296875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7265625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="13.54296875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="13.453125" style="36" customWidth="1"/>
+    <col min="18" max="18" width="12.54296875" style="36" customWidth="1"/>
+    <col min="19" max="19" width="21.453125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="20.1796875" style="31" customWidth="1"/>
+    <col min="21" max="21" width="18.7265625" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.7265625" style="36" customWidth="1"/>
+    <col min="25" max="25" width="12.81640625" style="36" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.7265625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="20.453125" style="31" customWidth="1"/>
     <col min="28" max="28" width="19" style="29" customWidth="1"/>
     <col min="29" max="29" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.28515625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="18.85546875" style="1" customWidth="1"/>
-    <col min="38" max="38" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.85546875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="24.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.26953125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="18.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="18.54296875" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.81640625" style="1" customWidth="1"/>
+    <col min="38" max="38" width="23.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.81640625" style="1" customWidth="1"/>
     <col min="40" max="40" width="13" style="33" customWidth="1"/>
     <col min="41" max="41" width="17" style="31" customWidth="1"/>
-    <col min="42" max="42" width="15.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="8.7109375" style="38" customWidth="1"/>
-    <col min="45" max="45" width="10.5703125" style="38" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.7265625" style="29" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="26.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.7265625" style="38" customWidth="1"/>
+    <col min="45" max="45" width="10.54296875" style="38" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="10" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="16.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="16.140625" style="39" customWidth="1"/>
-    <col min="49" max="49" width="9.140625" style="29"/>
-    <col min="50" max="16384" width="9.140625" style="1"/>
+    <col min="47" max="47" width="16.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="16.1796875" style="39" customWidth="1"/>
+    <col min="49" max="49" width="9.1796875" style="29"/>
+    <col min="50" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" s="5" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8688,7 +8696,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:49" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:49" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:AW2" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8704,49 +8712,49 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:AV2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.140625" style="25" customWidth="1"/>
-    <col min="14" max="15" width="20.140625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.1796875" style="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.1796875" style="25" customWidth="1"/>
+    <col min="14" max="15" width="20.1796875" style="3" customWidth="1"/>
+    <col min="16" max="16" width="11.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" style="3" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="20" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="25" customWidth="1"/>
-    <col min="28" max="28" width="20.42578125" style="3" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="24.7109375" style="3" customWidth="1"/>
-    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="38" max="41" width="18.85546875" style="3" customWidth="1"/>
-    <col min="42" max="42" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7265625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="20.453125" style="20" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.453125" style="25" customWidth="1"/>
+    <col min="28" max="28" width="20.453125" style="3" customWidth="1"/>
+    <col min="29" max="29" width="24.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="24.7265625" style="3" customWidth="1"/>
+    <col min="33" max="36" width="18.54296875" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="38" max="41" width="18.81640625" style="3" customWidth="1"/>
+    <col min="42" max="42" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="16.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="13" style="18" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="13" style="20" customWidth="1"/>
     <col min="47" max="47" width="17" style="25" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="16384" width="9.140625" style="3"/>
+    <col min="48" max="48" width="24.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:48" s="5" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8892,7 +8900,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:48" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:48" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:AV1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8909,23 +8917,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="7" customWidth="1"/>
-    <col min="2" max="3" width="25.7109375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="25.7109375" style="7" customWidth="1"/>
-    <col min="6" max="7" width="15.7109375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="26" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="25.7109375" style="7" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" style="7" customWidth="1"/>
-    <col min="13" max="13" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" style="7" customWidth="1"/>
+    <col min="2" max="3" width="25.7265625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="20.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="25.7265625" style="7" customWidth="1"/>
+    <col min="6" max="7" width="15.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" style="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.1796875" style="26" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="25.7265625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" style="7" customWidth="1"/>
+    <col min="13" max="13" width="16.7265625" style="7" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" style="7" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="7"/>
+    <col min="15" max="16384" width="9.1796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
@@ -8969,7 +8977,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8984,26 +8992,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="16" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" style="16" customWidth="1"/>
     <col min="2" max="2" width="12" style="16" customWidth="1"/>
     <col min="3" max="3" width="24" style="16" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" style="16" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="16" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.5703125" style="16" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="16" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="18.140625" style="16" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.7109375" style="17" customWidth="1"/>
-    <col min="16" max="16" width="20.7109375" style="23" customWidth="1"/>
-    <col min="17" max="17" width="20.7109375" style="28" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="16"/>
+    <col min="4" max="4" width="25.54296875" style="16" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" style="16" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.54296875" style="16" customWidth="1"/>
+    <col min="9" max="9" width="20.453125" style="16" customWidth="1"/>
+    <col min="10" max="10" width="18.1796875" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="18.1796875" style="16" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="10.7265625" style="17" customWidth="1"/>
+    <col min="16" max="16" width="20.7265625" style="23" customWidth="1"/>
+    <col min="17" max="17" width="20.7265625" style="28" customWidth="1"/>
+    <col min="18" max="16384" width="9.1796875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>146</v>
       </c>
@@ -9056,7 +9064,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="B1:Q2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9082,6 +9090,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9184,15 +9201,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
@@ -9211,6 +9219,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9227,12 +9243,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>